<commit_message>
[u] update add test case
</commit_message>
<xml_diff>
--- a/tests/ui_tests/post_login_report.xlsx
+++ b/tests/ui_tests/post_login_report.xlsx
@@ -452,7 +452,7 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-02 21:29:16</t>
+          <t>2026-04-12 16:44:24</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-04-02 21:29:20</t>
+          <t>2026-04-12 16:44:30</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-04-02 21:29:24</t>
+          <t>2026-04-12 16:44:36</t>
         </is>
       </c>
     </row>

</xml_diff>